<commit_message>
Fix printing, add delete student, photo upload and result export
</commit_message>
<xml_diff>
--- a/templates/student_upload_template.xlsx
+++ b/templates/student_upload_template.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valid Classes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="READ ME - How to fill" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,23 +28,29 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B6B6B"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002F5021"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00888888"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,12 +59,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F3D2E"/>
-        <bgColor rgb="000F3D2E"/>
+        <fgColor rgb="002F5021"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F6EE"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -65,17 +81,47 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFC8BC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFC8BC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFC8BC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFC8BC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,14 +490,14 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Student ID</t>
@@ -478,15 +524,15 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>AM0001</t>
+          <t>EXAMPLE-1</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Bello Fatima Ade</t>
+          <t>Amina Yusuf Example</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -501,16 +547,11 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2010-04-15</t>
+          <t>2011-05-20</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Male,Female"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -524,104 +565,177 @@
   <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Copy the exact class name from this list into the 'Class' column</t>
+          <t>Copy the exact class name below into the 'Class' column</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>الأوّل التّحضيريّ</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>الثّاني التّحضيريّ</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>الثّالث التّحضيريّ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>الأوّل الابتدائيّ</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>الثّاني الابتدائيّ</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>الثّالث الابتدائيّ</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>الرّابع الابتدائيّ</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>الأوّل الإعداديّ</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>الثّاني الإعداديّ</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>الثّالث الإعداديّ</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>الأوّل الثّانويّ</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>الثّاني الثّانويّ</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>الثّالث الثّانويّ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="95" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>HOW TO FILL THE BULK STUDENT UPLOAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>1.  Fill in the "Students" sheet only. Do NOT rename or delete the 5 column headers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>2.  Gender: type exactly Male or Female (capital M / capital F).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>3.  Class: copy the class name exactly as it appears in the "Valid Classes" sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>4.  Date of Birth: use the format YYYY-MM-DD  (example:  2012-08-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>5.  The yellow EXAMPLE rows are ignored automatically by the system when you upload - you can also just delete them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>6.  PHOTOS: Excel cannot carry photos. First upload this file, then open the "Students" page, click a student's card/profile and use "Add / Change Photo" to add each student's photo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>7.  When done, save the file as .xlsx and upload it on the "Add Student" page of the system.</t>
         </is>
       </c>
     </row>

</xml_diff>